<commit_message>
KG-206: added validation to optional parameters; updated excel template
</commit_message>
<xml_diff>
--- a/templates/GLL_excel_model.xlsx
+++ b/templates/GLL_excel_model.xlsx
@@ -22,24 +22,72 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="132">
   <si>
     <t xml:space="preserve">Color Codes Explained</t>
   </si>
   <si>
+    <t xml:space="preserve">Description</t>
+  </si>
+  <si>
     <t xml:space="preserve">Required</t>
   </si>
   <si>
+    <t xml:space="preserve">Strictly required property</t>
+  </si>
+  <si>
     <t xml:space="preserve">Optional</t>
   </si>
   <si>
+    <t xml:space="preserve">Optional property; Column name can not be re-used for user-defined data</t>
+  </si>
+  <si>
     <t xml:space="preserve">User Data [group]</t>
   </si>
   <si>
-    <t xml:space="preserve">Node Property</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Description</t>
+    <t xml:space="preserve">Add any user-defined property as a new column. For logical grouping, put your category in [brackets] (e.g. node property “property A” that belongs to the group “group A”).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data Types Explained</t>
+  </si>
+  <si>
+    <t xml:space="preserve">text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">any text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">number</t>
+  </si>
+  <si>
+    <t xml:space="preserve">whole decimal numbers or floating point numbers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">boolean</t>
+  </si>
+  <si>
+    <t xml:space="preserve">true or TRUE or 1, false or FALSE or 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RGBA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RGBA hex color code (e.g. #C33D3580 for 50% opacity) (last 2 digits are optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value 1 | value 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">List of categorical values of which one must be matched (excluding optional information in brackets)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">any</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Categorical view when text is given, slider-based view when numerical input is given</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Node Properties Explained</t>
   </si>
   <si>
     <t xml:space="preserve">Default Value</t>
@@ -66,18 +114,12 @@
     <t xml:space="preserve">Label of the node; if no Label is given, the ID is displayed per default</t>
   </si>
   <si>
-    <t xml:space="preserve">text</t>
-  </si>
-  <si>
     <t xml:space="preserve">Label Font Size</t>
   </si>
   <si>
     <t xml:space="preserve">Label font size</t>
   </si>
   <si>
-    <t xml:space="preserve">number</t>
-  </si>
-  <si>
     <t xml:space="preserve">Label Placement</t>
   </si>
   <si>
@@ -96,7 +138,7 @@
     <t xml:space="preserve">The color of the nodes label</t>
   </si>
   <si>
-    <t xml:space="preserve">RGBA hex color code</t>
+    <t xml:space="preserve">rgba</t>
   </si>
   <si>
     <t xml:space="preserve">Label Background Color</t>
@@ -156,13 +198,10 @@
     <t xml:space="preserve">property A [group A]</t>
   </si>
   <si>
-    <t xml:space="preserve">Add any user-defined node property as a new column. For logical grouping, put your category in [brackets] (e.g. node property “property A” that belongs to the group “group A”).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">any</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edge Property</t>
+    <t xml:space="preserve">User-defined node properties</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Edge Properties Explained</t>
   </si>
   <si>
     <t xml:space="preserve">Source ID</t>
@@ -186,15 +225,15 @@
     <t xml:space="preserve">center</t>
   </si>
   <si>
+    <t xml:space="preserve">The position of the label relative to the edge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#000000</t>
+  </si>
+  <si>
     <t xml:space="preserve">start | center | end</t>
   </si>
   <si>
-    <t xml:space="preserve">The position of the label relative to the edge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#000000</t>
-  </si>
-  <si>
     <t xml:space="preserve">The color of the edges label text</t>
   </si>
   <si>
@@ -222,9 +261,6 @@
     <t xml:space="preserve">Whether to automatically rotate the label to match the edge’s direction</t>
   </si>
   <si>
-    <t xml:space="preserve">boolean</t>
-  </si>
-  <si>
     <t xml:space="preserve">Color</t>
   </si>
   <si>
@@ -309,7 +345,7 @@
     <t xml:space="preserve">The stroke width of the halo</t>
   </si>
   <si>
-    <t xml:space="preserve">Add any user-defined edge property as a new column. Follows same logic as user-defined node properties.</t>
+    <t xml:space="preserve">User-defined edge properties</t>
   </si>
   <si>
     <t xml:space="preserve">my first numerical node property [group A]</t>
@@ -392,7 +428,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -423,6 +459,14 @@
     </font>
     <font>
       <b val="true"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
@@ -493,14 +537,14 @@
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top style="thin"/>
+      <top/>
       <bottom style="thin"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
-      <top/>
+      <top style="thin"/>
       <bottom style="thin"/>
       <diagonal/>
     </border>
@@ -530,7 +574,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -559,23 +603,55 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -583,11 +659,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -599,7 +671,7 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -814,18 +886,21 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="25.15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="141.43"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="15.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.06"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="136.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="15.13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="98.86"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
       </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -837,7 +912,10 @@
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
@@ -849,7 +927,10 @@
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -861,573 +942,646 @@
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" s="7"/>
+        <v>6</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="C4" s="8"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-      <c r="L4" s="7"/>
-      <c r="M4" s="7"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="s">
+      <c r="A6" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B6" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="10"/>
+      <c r="D6" s="11"/>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B7" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="C7" s="14"/>
+      <c r="D7" s="15"/>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="B8" s="13" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="C8" s="14"/>
+      <c r="D8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="1" t="s">
+      <c r="B9" s="13" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="C9" s="14"/>
+      <c r="D9" s="15"/>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B10" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="C10" s="14"/>
+      <c r="D10" s="15"/>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="16" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+      <c r="B11" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="C11" s="14"/>
+      <c r="D11" s="15"/>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="B12" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="C12" s="14"/>
+      <c r="D12" s="15"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+      <c r="B14" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C14" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="D14" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="12" t="s">
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+      <c r="B15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="C15" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="1" t="s">
+      <c r="D15" s="1" t="s">
         <v>27</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="D15" s="1" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>24</v>
+        <v>31</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" s="1" t="s">
-        <v>17</v>
+        <v>34</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C21" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="s">
+      <c r="B22" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B20" s="13" t="s">
+      <c r="C22" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" s="13" t="s">
+      <c r="D22" s="19" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="12"/>
-      <c r="C21" s="15"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="9" t="s">
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="s">
+      <c r="B23" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="C23" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C23" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
+      <c r="B24" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="12" t="s">
+      <c r="C24" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>14</v>
+      <c r="D24" s="20" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B25" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>14</v>
+      <c r="B25" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C26" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="11" t="s">
+      <c r="B26" s="1" t="s">
         <v>54</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B27" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="15" t="s">
+      <c r="B27" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="12" t="s">
-        <v>24</v>
+      <c r="C27" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
+      <c r="A28" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>58</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="20"/>
+      <c r="C29" s="22"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="C30" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C28" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D28" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="C29" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="D29" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
+      <c r="D30" s="17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="B30" s="12" t="s">
+      <c r="B31" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="C30" s="15" t="n">
+      <c r="C31" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C33" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C35" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D36" s="20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C37" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C38" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D30" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C31" s="15" t="n">
+      <c r="D38" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="C39" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D31" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="C32" s="16" t="n">
+      <c r="D39" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="C40" s="23" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D32" s="12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="C33" s="15" t="s">
-        <v>69</v>
-      </c>
-      <c r="D33" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="C34" s="15" t="n">
+      <c r="D40" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B41" s="20" t="s">
+        <v>80</v>
+      </c>
+      <c r="C41" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="D41" s="20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="22" t="n">
         <v>0.75</v>
       </c>
-      <c r="D34" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C35" s="15" t="n">
+      <c r="D42" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B43" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="D35" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D36" s="11" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C37" s="16" t="n">
+      <c r="D43" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B44" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="C44" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" s="19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B45" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="C45" s="23" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D37" s="12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="C38" s="15" t="n">
+      <c r="D45" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B46" s="20" t="s">
+        <v>92</v>
+      </c>
+      <c r="C46" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="D38" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C39" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D39" s="11" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="C40" s="16" t="n">
+      <c r="D46" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B47" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="C47" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="D47" s="19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B48" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="C48" s="23" t="n">
         <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
-      <c r="D40" s="12" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="C41" s="15" t="n">
+      <c r="D48" s="20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B49" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="C49" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="D41" s="17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="C42" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="D42" s="11" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B43" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="C43" s="16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D43" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B44" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="C44" s="15" t="n">
+      <c r="D49" s="24" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B50" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="C50" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="D50" s="19" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="B51" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="C51" s="23" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51" s="20" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B52" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C52" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="D44" s="12" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="C45" s="15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D45" s="12" t="s">
-        <v>45</v>
+      <c r="D52" s="20" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="B53" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C53" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D53" s="20" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1458,190 +1612,190 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="38.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="39.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.07"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="19" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="26" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>97</v>
+        <v>109</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>98</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="B2" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>101</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="E2" s="22" t="n">
+      <c r="A2" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>112</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>113</v>
+      </c>
+      <c r="D2" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="E2" s="29" t="n">
         <v>60</v>
       </c>
-      <c r="F2" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="G2" s="22" t="s">
-        <v>36</v>
-      </c>
-      <c r="H2" s="22" t="n">
+      <c r="F2" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="G2" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="H2" s="29" t="n">
         <v>150</v>
       </c>
-      <c r="I2" s="22" t="n">
+      <c r="I2" s="29" t="n">
         <v>150</v>
       </c>
-      <c r="J2" s="23" t="n">
+      <c r="J2" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="L2" s="23" t="n">
+      <c r="K2" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="L2" s="30" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="B3" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>107</v>
-      </c>
-      <c r="D3" s="21"/>
-      <c r="E3" s="22"/>
-      <c r="F3" s="22"/>
-      <c r="G3" s="22"/>
-      <c r="H3" s="22" t="n">
+      <c r="A3" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>118</v>
+      </c>
+      <c r="C3" s="28" t="s">
+        <v>119</v>
+      </c>
+      <c r="D3" s="28"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
+      <c r="H3" s="29" t="n">
         <v>-150</v>
       </c>
-      <c r="I3" s="22" t="n">
+      <c r="I3" s="29" t="n">
         <v>150</v>
       </c>
-      <c r="J3" s="23" t="n">
+      <c r="J3" s="30" t="n">
         <v>0.5</v>
       </c>
-      <c r="K3" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="L3" s="23" t="n">
+      <c r="K3" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="L3" s="30" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="C4" s="22" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22" t="n">
+      <c r="A4" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="29"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
+      <c r="H4" s="29" t="n">
         <v>450</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="29" t="n">
         <v>150</v>
       </c>
-      <c r="J4" s="23" t="n">
+      <c r="J4" s="30" t="n">
         <v>1.1</v>
       </c>
-      <c r="K4" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="L4" s="23" t="n">
+      <c r="K4" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="L4" s="30" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="23" t="n">
+      <c r="A5" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="C5" s="28" t="s">
+        <v>125</v>
+      </c>
+      <c r="D5" s="28"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="30" t="n">
         <v>1.3</v>
       </c>
-      <c r="K5" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="L5" s="23" t="n">
+      <c r="K5" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="L5" s="30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="B6" s="21"/>
-      <c r="C6" s="22"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="22"/>
-      <c r="I6" s="22"/>
-      <c r="J6" s="23" t="n">
+      <c r="A6" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="28"/>
+      <c r="C6" s="29"/>
+      <c r="D6" s="29"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
+      <c r="H6" s="29"/>
+      <c r="I6" s="29"/>
+      <c r="J6" s="30" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="L6" s="23" t="n">
+      <c r="K6" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="L6" s="30" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2703,125 +2857,125 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B2" s="27" t="s">
+        <v>117</v>
+      </c>
+      <c r="C2" s="28" t="s">
+        <v>131</v>
+      </c>
+      <c r="D2" s="28" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="G1" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="B2" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>119</v>
-      </c>
-      <c r="D2" s="21" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="F2" s="23" t="n">
+      <c r="F2" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="G2" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="H2" s="23" t="n">
+      <c r="G2" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="H2" s="30" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="B3" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="23" t="n">
+      <c r="A3" s="27" t="s">
+        <v>111</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="28"/>
+      <c r="D3" s="28"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="30" t="n">
         <v>0.5</v>
       </c>
-      <c r="G3" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="H3" s="23" t="n">
+      <c r="G3" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="H3" s="30" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
-        <v>108</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="23" t="n">
+      <c r="A4" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="30" t="n">
         <v>1.1</v>
       </c>
-      <c r="G4" s="23" t="s">
-        <v>104</v>
-      </c>
-      <c r="H4" s="23" t="n">
+      <c r="G4" s="30" t="s">
+        <v>116</v>
+      </c>
+      <c r="H4" s="30" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="B5" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="23" t="n">
+      <c r="A5" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="30" t="n">
         <v>1.3</v>
       </c>
-      <c r="G5" s="23" t="s">
-        <v>114</v>
-      </c>
-      <c r="H5" s="23" t="n">
+      <c r="G5" s="30" t="s">
+        <v>126</v>
+      </c>
+      <c r="H5" s="30" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="24"/>
-      <c r="G6" s="24"/>
-      <c r="H6" s="24"/>
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
KG-213: major style section revamp / cleanup / refactoring
</commit_message>
<xml_diff>
--- a/templates/GLL_excel_model.xlsx
+++ b/templates/GLL_excel_model.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="134">
   <si>
     <t xml:space="preserve">Color Codes Explained</t>
   </si>
@@ -108,6 +108,51 @@
     <t xml:space="preserve">text (unique)</t>
   </si>
   <si>
+    <t xml:space="preserve">Description of the node, displayed in the tooltip text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shape</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The shape of the node</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hexagon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">circle (●) | diamond (◆) | hexagon (⬢) | rect (■) | triangle (▲) | star (★)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The size of the node</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fill Color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The fill color of the node in RGBA format (e.g. #FF000080 for a red node with 50% opacity)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#C33D35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">rgba</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Border Size</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The stroke width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Border Color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The stroke color of the node in RGBA format</t>
+  </si>
+  <si>
     <t xml:space="preserve">Label</t>
   </si>
   <si>
@@ -138,51 +183,12 @@
     <t xml:space="preserve">The color of the nodes label</t>
   </si>
   <si>
-    <t xml:space="preserve">rgba</t>
-  </si>
-  <si>
     <t xml:space="preserve">Label Background Color</t>
   </si>
   <si>
     <t xml:space="preserve">Label background fill color</t>
   </si>
   <si>
-    <t xml:space="preserve">Description of the node, displayed in the tooltip text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Shape</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The shape of the node</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hexagon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">circle (●) | diamond (◆) | hexagon (⬢) | rect (■) | triangle (▲) | star (★)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Size</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The size of the node</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fill Color</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The fill color of the node in RGBA format (e.g. #FF000080 for a red node with 50% opacity)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#C33D35</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stroke Color</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The stroke color of the node in RGBA format</t>
-  </si>
-  <si>
     <t xml:space="preserve">X Coordinate</t>
   </si>
   <si>
@@ -216,6 +222,36 @@
     <t xml:space="preserve">The ID of the target node</t>
   </si>
   <si>
+    <t xml:space="preserve">The edge type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">line | cubic | quadratic | polyline</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Width</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The border width of the edge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line Dash</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The dash offset of the edge line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Color</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The stroke color of the edge in RGBA format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#403C5390</t>
+  </si>
+  <si>
     <t xml:space="preserve">Label of the edge; if no Label is given, the edge is only visible as line without any text</t>
   </si>
   <si>
@@ -234,6 +270,24 @@
     <t xml:space="preserve">start | center | end</t>
   </si>
   <si>
+    <t xml:space="preserve">Label Auto Rotate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Whether to automatically rotate the label to match the edge’s direction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Label Offset X</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The offset of the label on the X-Axis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Label Offset Y</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The offset of the label on the Y-Axis</t>
+  </si>
+  <si>
     <t xml:space="preserve">The color of the edges label text</t>
   </si>
   <si>
@@ -241,54 +295,6 @@
   </si>
   <si>
     <t xml:space="preserve">#E4E3EA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Label Offset X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The offset of the label on the X-Axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Label Offset Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The offset of the label on the Y-Axis</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Label Auto Rotate</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Whether to automatically rotate the label to match the edge’s direction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Color</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The stroke color of the edge in RGBA format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#403C5390</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Line Width</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The border width of the edge</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Line Dash</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The dash offset of the edge line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The edge type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">line</t>
-  </si>
-  <si>
-    <t xml:space="preserve">line | cubic | quadratic | polyline</t>
   </si>
   <si>
     <t xml:space="preserve">Start Arrow</t>
@@ -574,7 +580,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -633,10 +639,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -886,7 +888,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M54"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="29.06"/>
@@ -978,7 +980,6 @@
         <v>10</v>
       </c>
       <c r="C7" s="14"/>
-      <c r="D7" s="15"/>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
@@ -988,7 +989,6 @@
         <v>12</v>
       </c>
       <c r="C8" s="14"/>
-      <c r="D8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
@@ -998,7 +998,6 @@
         <v>14</v>
       </c>
       <c r="C9" s="14"/>
-      <c r="D9" s="15"/>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
@@ -1008,17 +1007,15 @@
         <v>16</v>
       </c>
       <c r="C10" s="14"/>
-      <c r="D10" s="15"/>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="15" t="s">
         <v>17</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="14"/>
-      <c r="D11" s="15"/>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="s">
@@ -1028,20 +1025,19 @@
         <v>20</v>
       </c>
       <c r="C12" s="14"/>
-      <c r="D12" s="15"/>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B14" s="17" t="s">
+      <c r="B14" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C14" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="17" t="s">
+      <c r="D14" s="16" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1061,10 +1057,10 @@
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>29</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>26</v>
@@ -1075,43 +1071,43 @@
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C17" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>11</v>
+      <c r="D17" s="18" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C18" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="D18" s="19" t="s">
-        <v>35</v>
+      <c r="C18" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="19" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1122,50 +1118,50 @@
       <c r="B20" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="D20" s="20" t="s">
-        <v>38</v>
+      <c r="C20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="19" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>1</v>
+        <v>41</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C21" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D21" s="1" t="s">
-        <v>9</v>
+      <c r="D21" s="19" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="19" t="s">
-        <v>45</v>
+        <v>26</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>47</v>
-      </c>
       <c r="C23" s="2" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>11</v>
@@ -1173,16 +1169,16 @@
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="C24" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="18" t="s">
         <v>50</v>
-      </c>
-      <c r="D24" s="20" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1195,7 +1191,7 @@
       <c r="C25" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D25" s="20" t="s">
+      <c r="D25" s="19" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1209,8 +1205,8 @@
       <c r="C26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D26" s="1" t="s">
-        <v>11</v>
+      <c r="D26" s="19" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1228,359 +1224,373 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C28" s="21" t="s">
+      <c r="C28" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D28" s="7" t="s">
+      <c r="D28" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="20"/>
-      <c r="C29" s="22"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" s="17" t="s">
+    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="19"/>
+      <c r="C30" s="21"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C30" s="18" t="s">
+      <c r="C31" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D30" s="17" t="s">
+      <c r="D31" s="16" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B31" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C31" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D31" s="20" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B32" s="20" t="s">
+      <c r="B32" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="20" t="s">
+      <c r="D32" s="19" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="B33" s="20" t="s">
+      <c r="A33" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="C33" s="22" t="s">
+      <c r="B33" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D33" s="20" t="s">
+      <c r="D33" s="19" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C34" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="0" t="s">
-        <v>11</v>
+      <c r="C34" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D34" s="18" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>67</v>
-      </c>
-      <c r="C35" s="22" t="s">
-        <v>68</v>
+        <v>69</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>70</v>
+      </c>
+      <c r="C35" s="21" t="n">
+        <v>0.75</v>
       </c>
       <c r="D35" s="19" t="s">
-        <v>69</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="B36" s="20" t="s">
-        <v>70</v>
-      </c>
-      <c r="C36" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="D36" s="20" t="s">
-        <v>38</v>
+        <v>71</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="C36" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="19" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B37" s="20" t="s">
-        <v>71</v>
-      </c>
-      <c r="C37" s="23" t="s">
-        <v>72</v>
-      </c>
-      <c r="D37" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="B37" s="19" t="s">
+        <v>74</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="D37" s="19" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="B38" s="20" t="s">
-        <v>74</v>
-      </c>
-      <c r="C38" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="20" t="s">
-        <v>11</v>
+        <v>43</v>
+      </c>
+      <c r="B38" s="19" t="s">
+        <v>76</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D38" s="19" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B39" s="20" t="s">
-        <v>76</v>
-      </c>
-      <c r="C39" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="B39" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="C39" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="D39" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B40" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="C40" s="23" t="n">
+        <v>47</v>
+      </c>
+      <c r="B40" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" s="18" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="B41" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="C41" s="22" t="n">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
-      <c r="D40" s="20" t="s">
+      <c r="D41" s="19" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B41" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="C41" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="D41" s="20" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="B42" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="C42" s="22" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D42" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B42" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C42" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="19" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="B43" s="20" t="s">
-        <v>85</v>
-      </c>
-      <c r="C43" s="22" t="n">
+        <v>86</v>
+      </c>
+      <c r="B43" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C43" s="21" t="n">
         <v>0</v>
       </c>
-      <c r="D43" s="20" t="s">
+      <c r="D43" s="19" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B44" s="20" t="s">
-        <v>86</v>
-      </c>
-      <c r="C44" s="22" t="s">
-        <v>87</v>
+        <v>51</v>
+      </c>
+      <c r="B44" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>26</v>
       </c>
       <c r="D44" s="19" t="s">
-        <v>88</v>
+        <v>38</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B45" s="19" t="s">
         <v>89</v>
       </c>
-      <c r="B45" s="20" t="s">
+      <c r="C45" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="C45" s="23" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="D45" s="20" t="s">
-        <v>13</v>
+      <c r="D45" s="19" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B46" s="20" t="s">
+      <c r="B46" s="19" t="s">
         <v>92</v>
       </c>
       <c r="C46" s="22" t="n">
-        <v>8</v>
-      </c>
-      <c r="D46" s="20" t="s">
-        <v>11</v>
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="19" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B47" s="20" t="s">
+      <c r="B47" s="19" t="s">
         <v>94</v>
       </c>
-      <c r="C47" s="23" t="s">
-        <v>95</v>
+      <c r="C47" s="21" t="n">
+        <v>8</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>96</v>
+        <v>11</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B48" s="19" t="s">
+        <v>96</v>
+      </c>
+      <c r="C48" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="B48" s="20" t="s">
+      <c r="D48" s="18" t="s">
         <v>98</v>
-      </c>
-      <c r="C48" s="23" t="n">
-        <f aca="false">FALSE()</f>
-        <v>0</v>
-      </c>
-      <c r="D48" s="20" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="B49" s="20" t="s">
+      <c r="B49" s="19" t="s">
         <v>100</v>
       </c>
       <c r="C49" s="22" t="n">
-        <v>8</v>
-      </c>
-      <c r="D49" s="24" t="s">
-        <v>11</v>
+        <f aca="false">FALSE()</f>
+        <v>0</v>
+      </c>
+      <c r="D49" s="19" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="B50" s="20" t="s">
+      <c r="B50" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="C50" s="23" t="s">
-        <v>95</v>
-      </c>
-      <c r="D50" s="19" t="s">
-        <v>96</v>
+      <c r="C50" s="21" t="n">
+        <v>8</v>
+      </c>
+      <c r="D50" s="23" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="B51" s="25" t="s">
+      <c r="B51" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="C51" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="D51" s="20" t="s">
-        <v>38</v>
+      <c r="C51" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="B52" s="25" t="s">
+      <c r="B52" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="C52" s="22" t="n">
+      <c r="C52" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="D52" s="19" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B53" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="C53" s="21" t="n">
         <v>3</v>
       </c>
-      <c r="D52" s="20" t="s">
+      <c r="D53" s="19" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B53" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="C53" s="22" t="s">
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="C54" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="D53" s="20" t="s">
+      <c r="D54" s="19" t="s">
         <v>19</v>
       </c>
     </row>
@@ -1600,7 +1610,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M1006"/>
+  <dimension ref="A1:P1006"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.2"/>
@@ -1612,7 +1622,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="38.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="39.17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="41.07"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="26" width="11.53"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="17" style="25" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1620,182 +1630,182 @@
         <v>24</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>46</v>
+        <v>33</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>51</v>
+        <v>41</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="J1" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B2" s="28" t="s">
-        <v>112</v>
-      </c>
-      <c r="C2" s="28" t="s">
+      <c r="A2" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="D2" s="28" t="s">
+      <c r="B2" s="27" t="s">
         <v>114</v>
       </c>
-      <c r="E2" s="29" t="n">
+      <c r="C2" s="27" t="s">
+        <v>115</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="E2" s="28" t="n">
         <v>60</v>
       </c>
-      <c r="F2" s="29" t="s">
-        <v>115</v>
-      </c>
-      <c r="G2" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="H2" s="29" t="n">
+      <c r="F2" s="28" t="s">
+        <v>117</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="H2" s="28" t="n">
         <v>150</v>
       </c>
-      <c r="I2" s="29" t="n">
+      <c r="I2" s="28" t="n">
         <v>150</v>
       </c>
-      <c r="J2" s="30" t="n">
+      <c r="J2" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="K2" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="L2" s="30" t="n">
+      <c r="K2" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="L2" s="29" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="3" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="B3" s="28" t="s">
+      <c r="A3" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="B3" s="27" t="s">
+        <v>120</v>
+      </c>
+      <c r="C3" s="27" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="27"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="28"/>
+      <c r="G3" s="28"/>
+      <c r="H3" s="28" t="n">
+        <v>-150</v>
+      </c>
+      <c r="I3" s="28" t="n">
+        <v>150</v>
+      </c>
+      <c r="J3" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K3" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="28" t="s">
-        <v>119</v>
-      </c>
-      <c r="D3" s="28"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
-      <c r="H3" s="29" t="n">
-        <v>-150</v>
-      </c>
-      <c r="I3" s="29" t="n">
+      <c r="L3" s="29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="28" t="s">
+        <v>124</v>
+      </c>
+      <c r="D4" s="28"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="28"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="28" t="n">
+        <v>450</v>
+      </c>
+      <c r="I4" s="28" t="n">
         <v>150</v>
       </c>
-      <c r="J3" s="30" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="K3" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="L3" s="30" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="28" t="s">
-        <v>121</v>
-      </c>
-      <c r="C4" s="29" t="s">
-        <v>122</v>
-      </c>
-      <c r="D4" s="29"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
-      <c r="H4" s="29" t="n">
-        <v>450</v>
-      </c>
-      <c r="I4" s="29" t="n">
-        <v>150</v>
-      </c>
-      <c r="J4" s="30" t="n">
+      <c r="J4" s="29" t="n">
         <v>1.1</v>
       </c>
-      <c r="K4" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="L4" s="30" t="n">
+      <c r="K4" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="L4" s="29" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="5" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="28" t="s">
-        <v>124</v>
-      </c>
-      <c r="C5" s="28" t="s">
+      <c r="A5" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="29"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="30" t="n">
+      <c r="B5" s="27" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5" s="27" t="s">
+        <v>127</v>
+      </c>
+      <c r="D5" s="27"/>
+      <c r="E5" s="28"/>
+      <c r="F5" s="28"/>
+      <c r="G5" s="28"/>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
+      <c r="J5" s="29" t="n">
         <v>1.3</v>
       </c>
-      <c r="K5" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="L5" s="30" t="n">
+      <c r="K5" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="L5" s="29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="B6" s="28"/>
-      <c r="C6" s="29"/>
-      <c r="D6" s="29"/>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="29"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="30" t="n">
+      <c r="A6" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="B6" s="27"/>
+      <c r="C6" s="28"/>
+      <c r="D6" s="28"/>
+      <c r="E6" s="28"/>
+      <c r="F6" s="28"/>
+      <c r="G6" s="28"/>
+      <c r="H6" s="28"/>
+      <c r="I6" s="28"/>
+      <c r="J6" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="K6" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="L6" s="30" t="n">
+      <c r="K6" s="29" t="s">
+        <v>128</v>
+      </c>
+      <c r="L6" s="29" t="n">
         <v>-1</v>
       </c>
     </row>
@@ -2738,61 +2748,501 @@
     <row r="943" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="944" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="945" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="946" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="947" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="948" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="949" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="950" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="951" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="952" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="953" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="954" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="955" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="956" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="957" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="958" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="959" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="960" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="961" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="962" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="963" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="964" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="965" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="966" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="967" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="968" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="969" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="970" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="971" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="972" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="973" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="974" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="975" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="976" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="977" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="978" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="979" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="980" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="981" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="982" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="983" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="984" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="985" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="986" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="987" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="988" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="989" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="990" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="991" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="992" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="993" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="994" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="995" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="996" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="997" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="998" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="999" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="1000" s="1" customFormat="true" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="946" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B946" s="1"/>
+      <c r="D946" s="1"/>
+      <c r="E946" s="1"/>
+      <c r="M946" s="1"/>
+      <c r="N946" s="1"/>
+      <c r="O946" s="1"/>
+      <c r="P946" s="1"/>
+    </row>
+    <row r="947" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B947" s="1"/>
+      <c r="D947" s="1"/>
+      <c r="E947" s="1"/>
+      <c r="M947" s="1"/>
+      <c r="N947" s="1"/>
+      <c r="O947" s="1"/>
+      <c r="P947" s="1"/>
+    </row>
+    <row r="948" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B948" s="1"/>
+      <c r="D948" s="1"/>
+      <c r="E948" s="1"/>
+      <c r="M948" s="1"/>
+      <c r="N948" s="1"/>
+      <c r="O948" s="1"/>
+      <c r="P948" s="1"/>
+    </row>
+    <row r="949" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B949" s="1"/>
+      <c r="D949" s="1"/>
+      <c r="E949" s="1"/>
+      <c r="M949" s="1"/>
+      <c r="N949" s="1"/>
+      <c r="O949" s="1"/>
+      <c r="P949" s="1"/>
+    </row>
+    <row r="950" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B950" s="1"/>
+      <c r="D950" s="1"/>
+      <c r="E950" s="1"/>
+      <c r="M950" s="1"/>
+      <c r="N950" s="1"/>
+      <c r="O950" s="1"/>
+      <c r="P950" s="1"/>
+    </row>
+    <row r="951" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B951" s="1"/>
+      <c r="D951" s="1"/>
+      <c r="E951" s="1"/>
+      <c r="M951" s="1"/>
+      <c r="N951" s="1"/>
+      <c r="O951" s="1"/>
+      <c r="P951" s="1"/>
+    </row>
+    <row r="952" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B952" s="1"/>
+      <c r="D952" s="1"/>
+      <c r="E952" s="1"/>
+      <c r="M952" s="1"/>
+      <c r="N952" s="1"/>
+      <c r="O952" s="1"/>
+      <c r="P952" s="1"/>
+    </row>
+    <row r="953" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B953" s="1"/>
+      <c r="D953" s="1"/>
+      <c r="E953" s="1"/>
+      <c r="M953" s="1"/>
+      <c r="N953" s="1"/>
+      <c r="O953" s="1"/>
+      <c r="P953" s="1"/>
+    </row>
+    <row r="954" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B954" s="1"/>
+      <c r="D954" s="1"/>
+      <c r="E954" s="1"/>
+      <c r="M954" s="1"/>
+      <c r="N954" s="1"/>
+      <c r="O954" s="1"/>
+      <c r="P954" s="1"/>
+    </row>
+    <row r="955" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B955" s="1"/>
+      <c r="D955" s="1"/>
+      <c r="E955" s="1"/>
+      <c r="M955" s="1"/>
+      <c r="N955" s="1"/>
+      <c r="O955" s="1"/>
+      <c r="P955" s="1"/>
+    </row>
+    <row r="956" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B956" s="1"/>
+      <c r="D956" s="1"/>
+      <c r="E956" s="1"/>
+      <c r="M956" s="1"/>
+      <c r="N956" s="1"/>
+      <c r="O956" s="1"/>
+      <c r="P956" s="1"/>
+    </row>
+    <row r="957" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B957" s="1"/>
+      <c r="D957" s="1"/>
+      <c r="E957" s="1"/>
+      <c r="M957" s="1"/>
+      <c r="N957" s="1"/>
+      <c r="O957" s="1"/>
+      <c r="P957" s="1"/>
+    </row>
+    <row r="958" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B958" s="1"/>
+      <c r="D958" s="1"/>
+      <c r="E958" s="1"/>
+      <c r="M958" s="1"/>
+      <c r="N958" s="1"/>
+      <c r="O958" s="1"/>
+      <c r="P958" s="1"/>
+    </row>
+    <row r="959" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B959" s="1"/>
+      <c r="D959" s="1"/>
+      <c r="E959" s="1"/>
+      <c r="M959" s="1"/>
+      <c r="N959" s="1"/>
+      <c r="O959" s="1"/>
+      <c r="P959" s="1"/>
+    </row>
+    <row r="960" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B960" s="1"/>
+      <c r="D960" s="1"/>
+      <c r="E960" s="1"/>
+      <c r="M960" s="1"/>
+      <c r="N960" s="1"/>
+      <c r="O960" s="1"/>
+      <c r="P960" s="1"/>
+    </row>
+    <row r="961" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B961" s="1"/>
+      <c r="D961" s="1"/>
+      <c r="E961" s="1"/>
+      <c r="M961" s="1"/>
+      <c r="N961" s="1"/>
+      <c r="O961" s="1"/>
+      <c r="P961" s="1"/>
+    </row>
+    <row r="962" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B962" s="1"/>
+      <c r="D962" s="1"/>
+      <c r="E962" s="1"/>
+      <c r="M962" s="1"/>
+      <c r="N962" s="1"/>
+      <c r="O962" s="1"/>
+      <c r="P962" s="1"/>
+    </row>
+    <row r="963" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B963" s="1"/>
+      <c r="D963" s="1"/>
+      <c r="E963" s="1"/>
+      <c r="M963" s="1"/>
+      <c r="N963" s="1"/>
+      <c r="O963" s="1"/>
+      <c r="P963" s="1"/>
+    </row>
+    <row r="964" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B964" s="1"/>
+      <c r="D964" s="1"/>
+      <c r="E964" s="1"/>
+      <c r="M964" s="1"/>
+      <c r="N964" s="1"/>
+      <c r="O964" s="1"/>
+      <c r="P964" s="1"/>
+    </row>
+    <row r="965" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B965" s="1"/>
+      <c r="D965" s="1"/>
+      <c r="E965" s="1"/>
+      <c r="M965" s="1"/>
+      <c r="N965" s="1"/>
+      <c r="O965" s="1"/>
+      <c r="P965" s="1"/>
+    </row>
+    <row r="966" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B966" s="1"/>
+      <c r="D966" s="1"/>
+      <c r="E966" s="1"/>
+      <c r="M966" s="1"/>
+      <c r="N966" s="1"/>
+      <c r="O966" s="1"/>
+      <c r="P966" s="1"/>
+    </row>
+    <row r="967" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B967" s="1"/>
+      <c r="D967" s="1"/>
+      <c r="E967" s="1"/>
+      <c r="M967" s="1"/>
+      <c r="N967" s="1"/>
+      <c r="O967" s="1"/>
+      <c r="P967" s="1"/>
+    </row>
+    <row r="968" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B968" s="1"/>
+      <c r="D968" s="1"/>
+      <c r="E968" s="1"/>
+      <c r="M968" s="1"/>
+      <c r="N968" s="1"/>
+      <c r="O968" s="1"/>
+      <c r="P968" s="1"/>
+    </row>
+    <row r="969" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B969" s="1"/>
+      <c r="D969" s="1"/>
+      <c r="E969" s="1"/>
+      <c r="M969" s="1"/>
+      <c r="N969" s="1"/>
+      <c r="O969" s="1"/>
+      <c r="P969" s="1"/>
+    </row>
+    <row r="970" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B970" s="1"/>
+      <c r="D970" s="1"/>
+      <c r="E970" s="1"/>
+      <c r="M970" s="1"/>
+      <c r="N970" s="1"/>
+      <c r="O970" s="1"/>
+      <c r="P970" s="1"/>
+    </row>
+    <row r="971" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B971" s="1"/>
+      <c r="D971" s="1"/>
+      <c r="E971" s="1"/>
+      <c r="M971" s="1"/>
+      <c r="N971" s="1"/>
+      <c r="O971" s="1"/>
+      <c r="P971" s="1"/>
+    </row>
+    <row r="972" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B972" s="1"/>
+      <c r="D972" s="1"/>
+      <c r="E972" s="1"/>
+      <c r="M972" s="1"/>
+      <c r="N972" s="1"/>
+      <c r="O972" s="1"/>
+      <c r="P972" s="1"/>
+    </row>
+    <row r="973" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B973" s="1"/>
+      <c r="D973" s="1"/>
+      <c r="E973" s="1"/>
+      <c r="M973" s="1"/>
+      <c r="N973" s="1"/>
+      <c r="O973" s="1"/>
+      <c r="P973" s="1"/>
+    </row>
+    <row r="974" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B974" s="1"/>
+      <c r="D974" s="1"/>
+      <c r="E974" s="1"/>
+      <c r="M974" s="1"/>
+      <c r="N974" s="1"/>
+      <c r="O974" s="1"/>
+      <c r="P974" s="1"/>
+    </row>
+    <row r="975" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B975" s="1"/>
+      <c r="D975" s="1"/>
+      <c r="E975" s="1"/>
+      <c r="M975" s="1"/>
+      <c r="N975" s="1"/>
+      <c r="O975" s="1"/>
+      <c r="P975" s="1"/>
+    </row>
+    <row r="976" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B976" s="1"/>
+      <c r="D976" s="1"/>
+      <c r="E976" s="1"/>
+      <c r="M976" s="1"/>
+      <c r="N976" s="1"/>
+      <c r="O976" s="1"/>
+      <c r="P976" s="1"/>
+    </row>
+    <row r="977" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B977" s="1"/>
+      <c r="D977" s="1"/>
+      <c r="E977" s="1"/>
+      <c r="M977" s="1"/>
+      <c r="N977" s="1"/>
+      <c r="O977" s="1"/>
+      <c r="P977" s="1"/>
+    </row>
+    <row r="978" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B978" s="1"/>
+      <c r="D978" s="1"/>
+      <c r="E978" s="1"/>
+      <c r="M978" s="1"/>
+      <c r="N978" s="1"/>
+      <c r="O978" s="1"/>
+      <c r="P978" s="1"/>
+    </row>
+    <row r="979" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B979" s="1"/>
+      <c r="D979" s="1"/>
+      <c r="E979" s="1"/>
+      <c r="M979" s="1"/>
+      <c r="N979" s="1"/>
+      <c r="O979" s="1"/>
+      <c r="P979" s="1"/>
+    </row>
+    <row r="980" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B980" s="1"/>
+      <c r="D980" s="1"/>
+      <c r="E980" s="1"/>
+      <c r="M980" s="1"/>
+      <c r="N980" s="1"/>
+      <c r="O980" s="1"/>
+      <c r="P980" s="1"/>
+    </row>
+    <row r="981" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B981" s="1"/>
+      <c r="D981" s="1"/>
+      <c r="E981" s="1"/>
+      <c r="M981" s="1"/>
+      <c r="N981" s="1"/>
+      <c r="O981" s="1"/>
+      <c r="P981" s="1"/>
+    </row>
+    <row r="982" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B982" s="1"/>
+      <c r="D982" s="1"/>
+      <c r="E982" s="1"/>
+      <c r="M982" s="1"/>
+      <c r="N982" s="1"/>
+      <c r="O982" s="1"/>
+      <c r="P982" s="1"/>
+    </row>
+    <row r="983" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B983" s="1"/>
+      <c r="D983" s="1"/>
+      <c r="E983" s="1"/>
+      <c r="M983" s="1"/>
+      <c r="N983" s="1"/>
+      <c r="O983" s="1"/>
+      <c r="P983" s="1"/>
+    </row>
+    <row r="984" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B984" s="1"/>
+      <c r="D984" s="1"/>
+      <c r="E984" s="1"/>
+      <c r="M984" s="1"/>
+      <c r="N984" s="1"/>
+      <c r="O984" s="1"/>
+      <c r="P984" s="1"/>
+    </row>
+    <row r="985" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B985" s="1"/>
+      <c r="D985" s="1"/>
+      <c r="E985" s="1"/>
+      <c r="M985" s="1"/>
+      <c r="N985" s="1"/>
+      <c r="O985" s="1"/>
+      <c r="P985" s="1"/>
+    </row>
+    <row r="986" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B986" s="1"/>
+      <c r="D986" s="1"/>
+      <c r="E986" s="1"/>
+      <c r="M986" s="1"/>
+      <c r="N986" s="1"/>
+      <c r="O986" s="1"/>
+      <c r="P986" s="1"/>
+    </row>
+    <row r="987" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B987" s="1"/>
+      <c r="D987" s="1"/>
+      <c r="E987" s="1"/>
+      <c r="M987" s="1"/>
+      <c r="N987" s="1"/>
+      <c r="O987" s="1"/>
+      <c r="P987" s="1"/>
+    </row>
+    <row r="988" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B988" s="1"/>
+      <c r="D988" s="1"/>
+      <c r="E988" s="1"/>
+      <c r="M988" s="1"/>
+      <c r="N988" s="1"/>
+      <c r="O988" s="1"/>
+      <c r="P988" s="1"/>
+    </row>
+    <row r="989" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B989" s="1"/>
+      <c r="D989" s="1"/>
+      <c r="E989" s="1"/>
+      <c r="M989" s="1"/>
+      <c r="N989" s="1"/>
+      <c r="O989" s="1"/>
+      <c r="P989" s="1"/>
+    </row>
+    <row r="990" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B990" s="1"/>
+      <c r="D990" s="1"/>
+      <c r="E990" s="1"/>
+      <c r="M990" s="1"/>
+      <c r="N990" s="1"/>
+      <c r="O990" s="1"/>
+      <c r="P990" s="1"/>
+    </row>
+    <row r="991" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B991" s="1"/>
+      <c r="D991" s="1"/>
+      <c r="E991" s="1"/>
+      <c r="M991" s="1"/>
+      <c r="N991" s="1"/>
+      <c r="O991" s="1"/>
+      <c r="P991" s="1"/>
+    </row>
+    <row r="992" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B992" s="1"/>
+      <c r="D992" s="1"/>
+      <c r="E992" s="1"/>
+      <c r="M992" s="1"/>
+      <c r="N992" s="1"/>
+      <c r="O992" s="1"/>
+      <c r="P992" s="1"/>
+    </row>
+    <row r="993" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B993" s="1"/>
+      <c r="D993" s="1"/>
+      <c r="E993" s="1"/>
+      <c r="M993" s="1"/>
+      <c r="N993" s="1"/>
+      <c r="O993" s="1"/>
+      <c r="P993" s="1"/>
+    </row>
+    <row r="994" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B994" s="1"/>
+      <c r="D994" s="1"/>
+      <c r="E994" s="1"/>
+      <c r="M994" s="1"/>
+      <c r="N994" s="1"/>
+      <c r="O994" s="1"/>
+      <c r="P994" s="1"/>
+    </row>
+    <row r="995" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B995" s="1"/>
+      <c r="D995" s="1"/>
+      <c r="E995" s="1"/>
+      <c r="M995" s="1"/>
+      <c r="N995" s="1"/>
+      <c r="O995" s="1"/>
+      <c r="P995" s="1"/>
+    </row>
+    <row r="996" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B996" s="1"/>
+      <c r="D996" s="1"/>
+      <c r="E996" s="1"/>
+      <c r="M996" s="1"/>
+      <c r="N996" s="1"/>
+      <c r="O996" s="1"/>
+      <c r="P996" s="1"/>
+    </row>
+    <row r="997" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B997" s="1"/>
+      <c r="D997" s="1"/>
+      <c r="E997" s="1"/>
+      <c r="M997" s="1"/>
+      <c r="N997" s="1"/>
+      <c r="O997" s="1"/>
+      <c r="P997" s="1"/>
+    </row>
+    <row r="998" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B998" s="1"/>
+      <c r="D998" s="1"/>
+      <c r="E998" s="1"/>
+      <c r="M998" s="1"/>
+      <c r="N998" s="1"/>
+      <c r="O998" s="1"/>
+      <c r="P998" s="1"/>
+    </row>
+    <row r="999" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B999" s="1"/>
+      <c r="D999" s="1"/>
+      <c r="E999" s="1"/>
+      <c r="M999" s="1"/>
+      <c r="N999" s="1"/>
+      <c r="O999" s="1"/>
+      <c r="P999" s="1"/>
+    </row>
+    <row r="1000" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B1000" s="1"/>
+      <c r="D1000" s="1"/>
+      <c r="E1000" s="1"/>
+      <c r="M1000" s="1"/>
+      <c r="N1000" s="1"/>
+      <c r="O1000" s="1"/>
+      <c r="P1000" s="1"/>
+    </row>
     <row r="1001" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1001" s="1"/>
       <c r="D1001" s="1"/>
@@ -2857,125 +3307,125 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>82</v>
+        <v>69</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="F1" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="G1" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="D2" s="27" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E2" s="27" t="s">
+        <v>118</v>
+      </c>
+      <c r="F2" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="H2" s="29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="26" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="27"/>
+      <c r="F3" s="29" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G3" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="H3" s="29" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
+        <v>122</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="27"/>
+      <c r="F4" s="29" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G4" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="H4" s="29" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" s="26" t="s">
+        <v>129</v>
+      </c>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="29" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G5" s="29" t="s">
         <v>128</v>
       </c>
-      <c r="G1" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="H1" s="6" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B2" s="27" t="s">
-        <v>117</v>
-      </c>
-      <c r="C2" s="28" t="s">
-        <v>131</v>
-      </c>
-      <c r="D2" s="28" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E2" s="28" t="s">
-        <v>116</v>
-      </c>
-      <c r="F2" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="H2" s="30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="27" t="s">
-        <v>111</v>
-      </c>
-      <c r="B3" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="C3" s="28"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="30" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G3" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="H3" s="30" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="27" t="s">
-        <v>120</v>
-      </c>
-      <c r="B4" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="C4" s="28"/>
-      <c r="D4" s="28"/>
-      <c r="E4" s="28"/>
-      <c r="F4" s="30" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="G4" s="30" t="s">
-        <v>116</v>
-      </c>
-      <c r="H4" s="30" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="27" t="s">
-        <v>123</v>
-      </c>
-      <c r="B5" s="27" t="s">
-        <v>127</v>
-      </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
-      <c r="E5" s="28"/>
-      <c r="F5" s="30" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="G5" s="30" t="s">
-        <v>126</v>
-      </c>
-      <c r="H5" s="30" t="n">
+      <c r="H5" s="29" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="31"/>
+      <c r="A6" s="19"/>
+      <c r="B6" s="19"/>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>